<commit_message>
Excel data updated by Sai Smitha
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,16 +5,20 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521741\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521752\Documents\project\test\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34A050C-05A1-4E12-850A-203DAF2F5BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C24D69C6-30A9-42EE-9655-8CC98DAE2D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="987" activeTab="5" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="TrainerRegistration" sheetId="2" r:id="rId2"/>
+    <sheet name="TrainerSeacrhBySkill" sheetId="3" r:id="rId3"/>
+    <sheet name="TrainerSearchByName" sheetId="4" r:id="rId4"/>
+    <sheet name="TrainerSearchByServiceLine" sheetId="5" r:id="rId5"/>
+    <sheet name="TrainerFilterByStatus" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="66">
   <si>
     <t>username</t>
   </si>
@@ -64,16 +68,198 @@
   </si>
   <si>
     <t>coach123</t>
+  </si>
+  <si>
+    <t>Full Name</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Skill Set</t>
+  </si>
+  <si>
+    <t>Experience</t>
+  </si>
+  <si>
+    <t>Available from</t>
+  </si>
+  <si>
+    <t>Available Till</t>
+  </si>
+  <si>
+    <t>Max Workload</t>
+  </si>
+  <si>
+    <t>Expected output</t>
+  </si>
+  <si>
+    <t>ramesh.c@cognizant.com</t>
+  </si>
+  <si>
+    <t>Java, SpringBoot</t>
+  </si>
+  <si>
+    <t>Validation failed</t>
+  </si>
+  <si>
+    <t>ramesh</t>
+  </si>
+  <si>
+    <t>Trainer added successfully</t>
+  </si>
+  <si>
+    <t>Rajesh</t>
+  </si>
+  <si>
+    <t>Python, Machine Learning</t>
+  </si>
+  <si>
+    <t>Pooja</t>
+  </si>
+  <si>
+    <t>Pooja@cognizant.com</t>
+  </si>
+  <si>
+    <t>Manu</t>
+  </si>
+  <si>
+    <t>manu@cognizant.com</t>
+  </si>
+  <si>
+    <t>Data Science, Python</t>
+  </si>
+  <si>
+    <t>Vaishnavi</t>
+  </si>
+  <si>
+    <t>vaishnavi@cognizant.com</t>
+  </si>
+  <si>
+    <t>Java, SpringBoot, SQL</t>
+  </si>
+  <si>
+    <t>Akash</t>
+  </si>
+  <si>
+    <t>akash@cognizant.com</t>
+  </si>
+  <si>
+    <t>Cobal</t>
+  </si>
+  <si>
+    <t>Mani</t>
+  </si>
+  <si>
+    <t>mani@cognizant.com</t>
+  </si>
+  <si>
+    <t>Python, ETL</t>
+  </si>
+  <si>
+    <t>Validation failed(start date&gt;end date)</t>
+  </si>
+  <si>
+    <t>Skill</t>
+  </si>
+  <si>
+    <t>Expected Output</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>java, spring</t>
+  </si>
+  <si>
+    <t>Shows 2 of 4 trainers list</t>
+  </si>
+  <si>
+    <t>Shows 1 of 4 trainers list</t>
+  </si>
+  <si>
+    <t>Shows empty list</t>
+  </si>
+  <si>
+    <t>Trainer name</t>
+  </si>
+  <si>
+    <t>Ramesh</t>
+  </si>
+  <si>
+    <t>Shows the trainer</t>
+  </si>
+  <si>
+    <t>Megha</t>
+  </si>
+  <si>
+    <t>Empty List</t>
+  </si>
+  <si>
+    <t>Service Line</t>
+  </si>
+  <si>
+    <t>QEA</t>
+  </si>
+  <si>
+    <t>Trainers list in QEA</t>
+  </si>
+  <si>
+    <t>ADM</t>
+  </si>
+  <si>
+    <t>Trainers list in ADM</t>
+  </si>
+  <si>
+    <t>XYZ</t>
+  </si>
+  <si>
+    <t>Empty list</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>All status</t>
+  </si>
+  <si>
+    <t>List of all trainers</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>List of available trainers</t>
+  </si>
+  <si>
+    <t>Unavailable</t>
+  </si>
+  <si>
+    <t>List of unavailable trainers</t>
+  </si>
+  <si>
+    <t>At capacity</t>
+  </si>
+  <si>
+    <t>List of trainers with at capacity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -96,13 +282,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -477,9 +667,431 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFBD520E-A90A-4D77-A289-1C5D578DC359}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="22.08984375" customWidth="1"/>
+    <col min="3" max="3" width="16.453125" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" customWidth="1"/>
+    <col min="7" max="7" width="12.90625" customWidth="1"/>
+    <col min="8" max="8" width="32.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2">
+        <v>46301</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46481</v>
+      </c>
+      <c r="G2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2">
+        <v>46343</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46454</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>46216</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46365</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2">
+        <v>46108</v>
+      </c>
+      <c r="F5" s="2">
+        <v>47378</v>
+      </c>
+      <c r="G5">
+        <v>-2</v>
+      </c>
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2">
+        <v>46188</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46481</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" s="2">
+        <v>46596</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46249</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9" s="2">
+        <v>46301</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46481</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{2DB78285-3B5E-455F-BA13-5FE1509852C1}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{8D8B936B-6B52-46D5-94F1-DC185C39AC4B}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{F31ADA34-7A54-4D20-AFE0-F8CF3B07F7A5}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{5A803497-EECE-49A9-9FE3-0B603F3FE8F6}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{0EE9BA74-B40F-4A45-BED9-4E555AF2AB0C}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{DC0898F4-C647-4169-9A6F-6E60AECACFB2}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{2EF9FE1F-0C9C-481F-8608-0CB3AF02D704}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6260E60-90EA-4FCE-A253-62CB9D4AD209}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="14.7265625" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D380A99-A520-44DA-A148-A421D5C7549C}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.7265625" customWidth="1"/>
+    <col min="2" max="2" width="22.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B08029B8-BC28-4487-B492-C3310B18E28E}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.26953125" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DF5EF28-01AC-47FE-8BC9-829DBAFA5B2A}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+    <col min="2" max="2" width="26.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel data updated by Ramya
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,20 +5,24 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521752\Documents\project\test\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521745\Project\Testing\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C24D69C6-30A9-42EE-9655-8CC98DAE2D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5DCD7C-0997-4A85-8DF4-34672DDB8C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="987" activeTab="5" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="987" firstSheet="1" activeTab="6" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="TrainerRegistration" sheetId="2" r:id="rId2"/>
     <sheet name="TrainerSeacrhBySkill" sheetId="3" r:id="rId3"/>
-    <sheet name="TrainerSearchByName" sheetId="4" r:id="rId4"/>
-    <sheet name="TrainerSearchByServiceLine" sheetId="5" r:id="rId5"/>
-    <sheet name="TrainerFilterByStatus" sheetId="6" r:id="rId6"/>
+    <sheet name="Cohort_Search_By_Coach" sheetId="7" r:id="rId4"/>
+    <sheet name="Cohort_Editing_By_Coach" sheetId="8" r:id="rId5"/>
+    <sheet name="CohortStatusfilter_By_Coach" sheetId="9" r:id="rId6"/>
+    <sheet name="Cohort_Creation" sheetId="10" r:id="rId7"/>
+    <sheet name="TrainerSearchByName" sheetId="4" r:id="rId8"/>
+    <sheet name="TrainerSearchByServiceLine" sheetId="5" r:id="rId9"/>
+    <sheet name="TrainerFilterByStatus" sheetId="6" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="131">
   <si>
     <t>username</t>
   </si>
@@ -242,13 +246,208 @@
   </si>
   <si>
     <t>List of trainers with at capacity</t>
+  </si>
+  <si>
+    <t>ADM26CS003</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>QEA26SD122</t>
+  </si>
+  <si>
+    <t>Shows Cohort</t>
+  </si>
+  <si>
+    <t>CohortCode_Or_Skill_Or_Trainer</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Nihar</t>
+  </si>
+  <si>
+    <t>Ramya</t>
+  </si>
+  <si>
+    <t>Shows 1 Cohort</t>
+  </si>
+  <si>
+    <t>Shows 2 cohorts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of Cohorts having java </t>
+  </si>
+  <si>
+    <t>JavaScript</t>
+  </si>
+  <si>
+    <t>Spring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of Cohorts having Spring </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of Trainees </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start Date </t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>Stream</t>
+  </si>
+  <si>
+    <t>Development</t>
+  </si>
+  <si>
+    <t>Expected Ouput</t>
+  </si>
+  <si>
+    <t>Cohort Created</t>
+  </si>
+  <si>
+    <t>Hyderabad</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Required_Skills</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>CS</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Spring,SQL</t>
+  </si>
+  <si>
+    <t>Cloud</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>SDET</t>
+  </si>
+  <si>
+    <t>MongoDB,React</t>
+  </si>
+  <si>
+    <t>Java,Spring</t>
+  </si>
+  <si>
+    <t>Assigned</t>
+  </si>
+  <si>
+    <t>Unassigned</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
+  </si>
+  <si>
+    <t>Cohorts List with Assigned Status</t>
+  </si>
+  <si>
+    <t>Cohorts List with Unassigned Status</t>
+  </si>
+  <si>
+    <t>Cohorts List with Pending Status</t>
+  </si>
+  <si>
+    <t>Cohorts List with Active Status</t>
+  </si>
+  <si>
+    <t>Cohorts List with Completed Status</t>
+  </si>
+  <si>
+    <t>Cohorts List with Cancelled Status</t>
+  </si>
+  <si>
+    <t>Cohort Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trainees Count </t>
+  </si>
+  <si>
+    <t>Required Skill(s)</t>
+  </si>
+  <si>
+    <t>Industry Vertical</t>
+  </si>
+  <si>
+    <t>Training Location</t>
+  </si>
+  <si>
+    <t>QEA26NF006</t>
+  </si>
+  <si>
+    <t>ADM26SD001</t>
+  </si>
+  <si>
+    <t>CS26CS004</t>
+  </si>
+  <si>
+    <t>ADM25CIS004</t>
+  </si>
+  <si>
+    <t>QEA24SD007</t>
+  </si>
+  <si>
+    <t>QEA26CIS001</t>
+  </si>
+  <si>
+    <t>CS26CS001</t>
+  </si>
+  <si>
+    <t>QEA26SD002</t>
+  </si>
+  <si>
+    <t>BFS</t>
+  </si>
+  <si>
+    <t>HC</t>
+  </si>
+  <si>
+    <t>INS</t>
+  </si>
+  <si>
+    <t>CS26CIS01</t>
+  </si>
+  <si>
+    <t>QEA26NF001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -263,6 +462,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F172A"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -286,10 +491,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -665,6 +871,60 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DF5EF28-01AC-47FE-8BC9-829DBAFA5B2A}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+    <col min="2" max="2" width="26.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFBD520E-A90A-4D77-A289-1C5D578DC359}">
   <dimension ref="A1:H9"/>
@@ -959,6 +1219,816 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6147596-CEDE-4F32-9E23-F0F5EC0F6198}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="31.90625" customWidth="1"/>
+    <col min="2" max="2" width="26.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22E8E1F5-A43C-412B-8DF7-12CCA85343A2}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.7265625" customWidth="1"/>
+    <col min="2" max="2" width="22.453125" customWidth="1"/>
+    <col min="3" max="3" width="18.90625" customWidth="1"/>
+    <col min="4" max="4" width="18.08984375" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="6" width="15.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.54296875" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2">
+        <v>46297</v>
+      </c>
+      <c r="D2" s="2">
+        <v>46387</v>
+      </c>
+      <c r="E2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46248</v>
+      </c>
+      <c r="D3" s="2">
+        <v>46295</v>
+      </c>
+      <c r="E3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B4">
+        <v>20</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46248</v>
+      </c>
+      <c r="D4" s="2">
+        <v>46387</v>
+      </c>
+      <c r="E4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5">
+        <v>35</v>
+      </c>
+      <c r="C5" s="2">
+        <v>45803</v>
+      </c>
+      <c r="D5" s="2">
+        <v>45767</v>
+      </c>
+      <c r="E5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2">
+        <v>45351</v>
+      </c>
+      <c r="D6" s="2">
+        <v>45442</v>
+      </c>
+      <c r="E6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46297</v>
+      </c>
+      <c r="D7" s="2">
+        <v>46417</v>
+      </c>
+      <c r="E7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" t="s">
+        <v>96</v>
+      </c>
+      <c r="H7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2">
+        <v>45803</v>
+      </c>
+      <c r="D8" s="2">
+        <v>45895</v>
+      </c>
+      <c r="E8" t="s">
+        <v>84</v>
+      </c>
+      <c r="F8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46037</v>
+      </c>
+      <c r="D9" s="2">
+        <v>46137</v>
+      </c>
+      <c r="E9" t="s">
+        <v>89</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
+        <v>98</v>
+      </c>
+      <c r="H9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46288</v>
+      </c>
+      <c r="D10" s="2">
+        <v>46384</v>
+      </c>
+      <c r="F10" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" t="s">
+        <v>94</v>
+      </c>
+      <c r="H10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F3AF794-2849-41E4-A829-E831BBFED114}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
+    <col min="2" max="2" width="45.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3E81392-D90F-4046-B97E-C3FC36D72449}">
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="13.453125" customWidth="1"/>
+    <col min="3" max="3" width="19.90625" customWidth="1"/>
+    <col min="4" max="4" width="14.90625" customWidth="1"/>
+    <col min="5" max="5" width="18.90625" customWidth="1"/>
+    <col min="6" max="6" width="14.08984375" customWidth="1"/>
+    <col min="7" max="7" width="18.1796875" customWidth="1"/>
+    <col min="8" max="8" width="17.08984375" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" customWidth="1"/>
+    <col min="10" max="10" width="15.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" t="s">
+        <v>116</v>
+      </c>
+      <c r="I1" t="s">
+        <v>117</v>
+      </c>
+      <c r="J1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46297</v>
+      </c>
+      <c r="G2" s="2">
+        <v>46387</v>
+      </c>
+      <c r="H2" t="s">
+        <v>126</v>
+      </c>
+      <c r="I2" t="s">
+        <v>84</v>
+      </c>
+      <c r="J2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46248</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46295</v>
+      </c>
+      <c r="H3" t="s">
+        <v>127</v>
+      </c>
+      <c r="I3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46248</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46387</v>
+      </c>
+      <c r="H4" t="s">
+        <v>128</v>
+      </c>
+      <c r="I4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5">
+        <v>35</v>
+      </c>
+      <c r="C5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="2">
+        <v>45803</v>
+      </c>
+      <c r="G5" s="2">
+        <v>45767</v>
+      </c>
+      <c r="H5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I5" t="s">
+        <v>84</v>
+      </c>
+      <c r="J5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="2">
+        <v>45351</v>
+      </c>
+      <c r="G6" s="2">
+        <v>45442</v>
+      </c>
+      <c r="H6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" t="s">
+        <v>89</v>
+      </c>
+      <c r="J6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46297</v>
+      </c>
+      <c r="G7" s="2">
+        <v>46417</v>
+      </c>
+      <c r="H7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B8">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F8" s="2">
+        <v>45803</v>
+      </c>
+      <c r="G8" s="2">
+        <v>45895</v>
+      </c>
+      <c r="H8" t="s">
+        <v>126</v>
+      </c>
+      <c r="I8" t="s">
+        <v>84</v>
+      </c>
+      <c r="J8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46037</v>
+      </c>
+      <c r="G9" s="2">
+        <v>46137</v>
+      </c>
+      <c r="H9" t="s">
+        <v>128</v>
+      </c>
+      <c r="I9" t="s">
+        <v>89</v>
+      </c>
+      <c r="J9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F10" s="2">
+        <v>46300</v>
+      </c>
+      <c r="G10" s="2">
+        <v>46417</v>
+      </c>
+      <c r="H10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I10" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B11">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46251</v>
+      </c>
+      <c r="G11" s="2">
+        <v>46351</v>
+      </c>
+      <c r="I11" t="s">
+        <v>84</v>
+      </c>
+      <c r="J11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B12">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" t="s">
+        <v>90</v>
+      </c>
+      <c r="F12" s="2">
+        <v>46145</v>
+      </c>
+      <c r="G12" s="2">
+        <v>46238</v>
+      </c>
+      <c r="H12" t="s">
+        <v>126</v>
+      </c>
+      <c r="J12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D380A99-A520-44DA-A148-A421D5C7549C}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -996,7 +2066,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B08029B8-BC28-4487-B492-C3310B18E28E}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1040,58 +2110,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DF5EF28-01AC-47FE-8BC9-829DBAFA5B2A}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="13.26953125" customWidth="1"/>
-    <col min="2" max="2" width="26.81640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel data updated by Nihar
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521745\Project\Testing\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521739\IdeaProjects\trainmate-test\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5DCD7C-0997-4A85-8DF4-34672DDB8C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D4487C-5353-4917-99F2-02CFF33F9D57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="987" firstSheet="1" activeTab="6" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" tabRatio="987" firstSheet="6" activeTab="10" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="TrainerSearchByName" sheetId="4" r:id="rId8"/>
     <sheet name="TrainerSearchByServiceLine" sheetId="5" r:id="rId9"/>
     <sheet name="TrainerFilterByStatus" sheetId="6" r:id="rId10"/>
+    <sheet name="Cohort_or_Skill_SearchByTrainer" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="140">
   <si>
     <t>username</t>
   </si>
@@ -441,6 +442,33 @@
   </si>
   <si>
     <t>QEA26NF001</t>
+  </si>
+  <si>
+    <t>QEA26SD009</t>
+  </si>
+  <si>
+    <t>QEA26SD004</t>
+  </si>
+  <si>
+    <t>Java, Spring Boot</t>
+  </si>
+  <si>
+    <t>QEA26SD010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shows Cohort </t>
+  </si>
+  <si>
+    <t>SQL,python</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QEA26SD939	</t>
+  </si>
+  <si>
+    <t>List of cohort having Java, Spring Boot</t>
+  </si>
+  <si>
+    <t>CohortCode_or_Skill</t>
   </si>
 </sst>
 </file>
@@ -925,6 +953,76 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F4C8015-4043-4E04-B91F-D43B3C5C473F}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.36328125" customWidth="1"/>
+    <col min="2" max="2" width="30.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFBD520E-A90A-4D77-A289-1C5D578DC359}">
   <dimension ref="A1:H9"/>

</xml_diff>

<commit_message>
excel data updated by Chavi
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521739\IdeaProjects\trainmate-test\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521741\Idea projects\TrainMate_test\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D4487C-5353-4917-99F2-02CFF33F9D57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F500DD-BB76-4A50-AEB8-69C6FD3E924D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" tabRatio="987" firstSheet="6" activeTab="10" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="987" xr2:uid="{485C5688-5C9D-403B-9130-D22C3FB88A97}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="TrainerRegistration" sheetId="2" r:id="rId2"/>
-    <sheet name="TrainerSeacrhBySkill" sheetId="3" r:id="rId3"/>
+    <sheet name="TrainerSearchBySkill" sheetId="3" r:id="rId3"/>
     <sheet name="Cohort_Search_By_Coach" sheetId="7" r:id="rId4"/>
     <sheet name="Cohort_Editing_By_Coach" sheetId="8" r:id="rId5"/>
     <sheet name="CohortStatusfilter_By_Coach" sheetId="9" r:id="rId6"/>
@@ -24,6 +24,9 @@
     <sheet name="TrainerSearchByServiceLine" sheetId="5" r:id="rId9"/>
     <sheet name="TrainerFilterByStatus" sheetId="6" r:id="rId10"/>
     <sheet name="Cohort_or_Skill_SearchByTrainer" sheetId="11" r:id="rId11"/>
+    <sheet name="Cohort_Search_By_Admin" sheetId="12" r:id="rId12"/>
+    <sheet name="CohortStatusfilter_By_Admin" sheetId="13" r:id="rId13"/>
+    <sheet name="CohortSLfilter_By_Admin" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="147">
   <si>
     <t>username</t>
   </si>
@@ -469,6 +472,27 @@
   </si>
   <si>
     <t>CohortCode_or_Skill</t>
+  </si>
+  <si>
+    <t>CohortCode_Or_Skill_Or_Trainer_Or_Coach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amit </t>
+  </si>
+  <si>
+    <t>Shows 6 cohorts</t>
+  </si>
+  <si>
+    <t>Processing</t>
+  </si>
+  <si>
+    <t>Cohorts List with Processing Status</t>
+  </si>
+  <si>
+    <t>Cohorts List with ADM Service Line</t>
+  </si>
+  <si>
+    <t>Cohorts List with QEA Service Line</t>
   </si>
 </sst>
 </file>
@@ -1023,6 +1047,216 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E5DAE2-3E92-4CE0-A5DB-0964450C0891}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="36.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89D1AE2A-4673-46E5-A0D2-BC5AA89E028F}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
+    <col min="2" max="2" width="45.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C4C0A3E-5945-4326-BFA5-60427829EF5C}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.26953125" customWidth="1"/>
+    <col min="2" max="2" width="45.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFBD520E-A90A-4D77-A289-1C5D578DC359}">
   <dimension ref="A1:H9"/>

</xml_diff>